<commit_message>
🚀 Final polish: UI/UX updates + minor fixes
</commit_message>
<xml_diff>
--- a/xlsx/RESOURCE_UPLOADER.xlsx
+++ b/xlsx/RESOURCE_UPLOADER.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,6 +460,870 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Case-Study-All-Chapters_1mTuOHG3ah_AJ6kfdLciyumFMTOj50b78.pdf</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/case_based_questions/Case-Study-All-Chapters_1mTuOHG3ah_AJ6kfdLciyumFMTOj50b78.pdf</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Case Study (All Chapters)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Case Based Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>case_based_questions</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Basic-2024-2025-with-Solution_1AKPa-z8EfdV6zrV7iLBrlJ_PYlZh1nMX.pdf</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/sample_papers/Basic-2024-2025-with-Solution_1AKPa-z8EfdV6zrV7iLBrlJ_PYlZh1nMX.pdf</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Basic (2024-2025) With Solution</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sample Papers for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>sample_papers</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Standard-2024-2025-with-solution_13vras5PqieLebe_nLadoHUr6dlGksPK7.pdf</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/sample_papers/Standard-2024-2025-with-solution_13vras5PqieLebe_nLadoHUr6dlGksPK7.pdf</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Standard (2024-2025) With Solution</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sample Papers for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>sample_papers</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CH-1-Real-Number_1KEjd1PtHmhECYmtIVAIMzdCmLCfRS0jT.pdf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-1-Real-Number_1KEjd1PtHmhECYmtIVAIMzdCmLCfRS0jT.pdf</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Ch 1 - Real Number</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CH-2-Polynomials_1a_AQAjO0fnGB_tASwoy7QbvVqv8ypo2M.pdf</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-2-Polynomials_1a_AQAjO0fnGB_tASwoy7QbvVqv8ypo2M.pdf</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ch 2 - Polynomials</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CH-3-Pair-of-Linear-Equations-in-Two-Variables_13rZw4nDD7LV9hXhYi5J-2uCvsrRWU7ZZ.pdf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-3-Pair-of-Linear-Equations-in-Two-Variables_13rZw4nDD7LV9hXhYi5J-2uCvsrRWU7ZZ.pdf</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Ch 3 - Pair Of Linear Equations In Two Variables</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CH-4-Quadratic-Equation_1vhZG00hT90c2-0FEWU2C57EpQlb4pLSa.pdf</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-4-Quadratic-Equation_1vhZG00hT90c2-0FEWU2C57EpQlb4pLSa.pdf</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ch 4 - Quadratic Equation</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CH-5-Arithmetic-Progression_11V7i3_2sJ7RZNstTXbjlFrX0sanN3MZ9.pdf</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-5-Arithmetic-Progression_11V7i3_2sJ7RZNstTXbjlFrX0sanN3MZ9.pdf</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Ch 5 - Arithmetic Progression</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CH-6-Triangles_1dP3TFuMNxz9I25O1s2RDbeG0GKQ_Y_Nf.pdf</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-6-Triangles_1dP3TFuMNxz9I25O1s2RDbeG0GKQ_Y_Nf.pdf</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Ch 6 - Triangles</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CH-7-Coordinate-Geometry_1e-dNaC2Skk9-dta6SNLvof-kpZC3Aswd.pdf</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-7-Coordinate-Geometry_1e-dNaC2Skk9-dta6SNLvof-kpZC3Aswd.pdf</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ch 7 - Coordinate Geometry</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CH-8-Trigonometry_1nsH_Go7nxXasSX0HWoYSad9aUCl-vDfO.pdf</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-8-Trigonometry_1nsH_Go7nxXasSX0HWoYSad9aUCl-vDfO.pdf</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ch 8 - Trigonometry</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CH-9-Applications-of-Trigonometry_1oTnQH30HPoBKEHOicZ0c7MXrDP4GduGg.pdf</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-9-Applications-of-Trigonometry_1oTnQH30HPoBKEHOicZ0c7MXrDP4GduGg.pdf</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ch 9 - Applications Of Trigonometry</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CH-10-Circles_1CC5TaIgJTR3ZuB6BHUDmWIXYDmZ2_VAo.pdf</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-10-Circles_1CC5TaIgJTR3ZuB6BHUDmWIXYDmZ2_VAo.pdf</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ch 10 - Circles</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CH-11-Areas-Related-to-Circles_1NGuipqjtxnpArlQZtddD88C1rC2dyFzB.pdf</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-11-Areas-Related-to-Circles_1NGuipqjtxnpArlQZtddD88C1rC2dyFzB.pdf</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ch 11 - Areas Related To Circles</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CH-12-Surface-Areas-Volumes_1oS693cOTkYhY8PUn5w-NDBf9mL_mCa86.pdf</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-12-Surface-Areas-Volumes_1oS693cOTkYhY8PUn5w-NDBf9mL_mCa86.pdf</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Ch 12 - Surface Areas &amp; Volumes</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CH-13-Statistics_1WblRmjMTLvxwsF-y3_9KECE8Xh51qIpu.pdf</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-13-Statistics_1WblRmjMTLvxwsF-y3_9KECE8Xh51qIpu.pdf</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Ch 13 - Statistics</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CH-14-Probability_1jRVyAa184Jz-FxxuDDguZMJPkxCZymUf.pdf</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/CH-14-Probability_1jRVyAa184Jz-FxxuDDguZMJPkxCZymUf.pdf</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ch 14 - Probability</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Polynomials-Worksheet-UNLOCKED_1ZgUSqxEoH3KnobfrlOKtsQGzCHfoC_cM.pdf</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/Polynomials-Worksheet-UNLOCKED_1ZgUSqxEoH3KnobfrlOKtsQGzCHfoC_cM.pdf</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Polynomials - Worksheet (Unlocked)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Triangles-Worksheet-UNLOCKED_11SIma-Eu2ljYlWAKSFpS04tCyqAjij7z.pdf</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/Triangles-Worksheet-UNLOCKED_11SIma-Eu2ljYlWAKSFpS04tCyqAjij7z.pdf</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Triangles - Worksheet (Unlocked)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Probability-Worksheet-UNLOCKED_1iluMHbcoJX73DZe-oe7-a500yv7OHiAB.pdf</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>bulk_upload_resources/class_10_standard/previous_year_questions/Probability-Worksheet-UNLOCKED_1iluMHbcoJX73DZe-oe7-a500yv7OHiAB.pdf</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Probability - Worksheet (Unlocked)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Previous Year Questions for Class 10 Standard</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>previous_year_questions</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>class_10_standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Sample-Paper-1_Class9.pdf</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>uploads/study_materials/Sample-Paper-1_Class9.pdf</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Sample Paper 1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Class 9 Sample Papers</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>worksheet</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>class_9</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sample-Paper-2_Class9.pdf</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>uploads/study_materials/Sample-Paper-2_Class9.pdf</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Sample Paper 2</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Class 9 Sample Papers</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>worksheet</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>class_9</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sample-Paper-3_Class9.pdf</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>uploads/study_materials/Sample-Paper-3_Class9.pdf</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Sample Paper 3</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Class 9 Sample Papers</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>worksheet</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>class_9</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Chapter-wise-Notes_Class9.pdf</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>uploads/study_materials/Chapter-wise-Notes_Class9.pdf</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Chapter wise Notes</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Class 9 Notes</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>pyq</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>class_9</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Lines-Angles-Worksheet_Class9.pdf</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>uploads/study_materials/Lines-Angles-Worksheet_Class9.pdf</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Lines &amp; Angles - Worksheet</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Class 9 Worksheets</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>worksheet</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>class_9</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Herons-Formula-Worksheet_Class9.pdf</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>uploads/study_materials/Herons-Formula-Worksheet_Class9.pdf</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Heron's Formula - Worksheet</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Class 9 Worksheets</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>worksheet</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>class_9</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>IMP-Questions-NCERT_Class9.xlsx</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>uploads/study_materials/IMP-Questions-NCERT_Class9.xlsx</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CLASS IX I.M.P's (NCERT) -SEC</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Class 9 Important Questions</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>pyq</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>class_9</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>